<commit_message>
Add reviewed nine-school follow-up profiles and precise combined guidance display
</commit_message>
<xml_diff>
--- a/site/exports/hust-cs-storage.xlsx
+++ b/site/exports/hust-cs-storage.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rc34d1e2d587b465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R3add24c2459d42b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R2c5f358e46e74287"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="Rfda5237fdd444d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R987f525a2422446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Red7fe892901748b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R41ccf298736c42a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Ree381e095b7448c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R744d52452ee843e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Redd39847bfe94930"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T19_0" displayName="T19_0" ref="A1:K2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T19_0" displayName="T19_0" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
@@ -158,7 +158,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T19_1" displayName="T19_1" ref="A1:S6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T19_1" displayName="T19_1" ref="A1:S21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
@@ -185,7 +185,27 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T19_3" displayName="T19_3" ref="A1:L2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T19_2" displayName="T19_2" ref="A1:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="姓名"/>
+    <x:tableColumn id="2" name="导师姓名"/>
+    <x:tableColumn id="3" name="关系类型"/>
+    <x:tableColumn id="4" name="阶段"/>
+    <x:tableColumn id="5" name="简介"/>
+    <x:tableColumn id="6" name="在职状态"/>
+    <x:tableColumn id="7" name="状态说明"/>
+    <x:tableColumn id="8" name="已核在职主页"/>
+    <x:tableColumn id="9" name="关系来源"/>
+    <x:tableColumn id="10" name="任职来源"/>
+    <x:tableColumn id="11" name="所属学校ID"/>
+    <x:tableColumn id="12" name="所属学校"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T19_3" displayName="T19_3" ref="A1:L5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
@@ -204,8 +224,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T19_4" displayName="T19_4" ref="A1:G5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T19_4" displayName="T19_4" ref="A1:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -495,10 +515,109 @@
         <x:v>华中科技大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" ht="64" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>计算机科学与技术学院·存储所</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str"/>
+      <x:c r="E3" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>导师现职未核，未知不展示已核在岗导航。；精选论文非全集。；本科及导师未披露；硕士起讫表与简介冲突。</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str">
+        <x:v>个人页当前不可达或正文未核；保留既有分级职业证据，不重试受限来源</x:v>
+      </x:c>
+      <x:c r="I3" s="6" t="str">
+        <x:v>学校官方英文职业简介（独立可读来源）：https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="64" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>计算机科学与技术学院·存储所</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="E4" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>导师现职未核，未知不展示已核在岗导航。；精选论文非全集。</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I4" s="6" t="str"/>
+      <x:c r="J4" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>计算机科学与技术学院·存储所</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>导师现职未核，未知不展示已核在岗导航。；精选论文非全集。；校内主页请求超时，未冒称已读校内履历；本科院校历史名称与法人属性待核。</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str">
+        <x:v>本人公开职业网站；学校门户超时，非校内正文实读</x:v>
+      </x:c>
+      <x:c r="I5" s="6" t="str"/>
+      <x:c r="J5" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a04b328eff14b06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb76bcae85b1d4781"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -818,10 +937,729 @@
         <x:v>华中科技大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str"/>
+      <x:c r="F7" s="6" t="str">
+        <x:v>1999</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str"/>
+      <x:c r="H7" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I7" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L7" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M7" s="7" t="str"/>
+      <x:c r="N7" s="6" t="str"/>
+      <x:c r="O7" s="6" t="str">
+        <x:v>简介明确1999获硕士；同页教育表却将硕士写为1999.09–2003.12，冲突保留，end取明确获授年。</x:v>
+      </x:c>
+      <x:c r="P7" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q7" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="R7" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S7" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>1999-09</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>2003-12</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str"/>
+      <x:c r="H8" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I8" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L8" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M8" s="7" t="str"/>
+      <x:c r="N8" s="6" t="str"/>
+      <x:c r="O8" s="6" t="str">
+        <x:v>简介明确2003获博士；教育表结束月不当授位月。</x:v>
+      </x:c>
+      <x:c r="P8" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q8" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="R8" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S8" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>副教授</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>华中科技大学计算机科学与技术学院</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str"/>
+      <x:c r="F9" s="6" t="str"/>
+      <x:c r="G9" s="6" t="str"/>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str"/>
+      <x:c r="J9" s="6" t="str"/>
+      <x:c r="K9" s="6" t="str"/>
+      <x:c r="L9" s="6" t="str"/>
+      <x:c r="M9" s="7" t="str"/>
+      <x:c r="N9" s="6" t="str"/>
+      <x:c r="O9" s="6" t="str"/>
+      <x:c r="P9" s="6" t="str"/>
+      <x:c r="Q9" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="R9" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S9" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>任职（未注明当时职称）</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>华中科技大学计算机科学与技术学院</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>1999-09</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str"/>
+      <x:c r="G10" s="6" t="str"/>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str"/>
+      <x:c r="J10" s="6" t="str"/>
+      <x:c r="K10" s="6" t="str"/>
+      <x:c r="L10" s="6" t="str"/>
+      <x:c r="M10" s="7" t="str"/>
+      <x:c r="N10" s="6" t="str"/>
+      <x:c r="O10" s="6" t="str"/>
+      <x:c r="P10" s="6" t="str"/>
+      <x:c r="Q10" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="R10" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S10" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>2007-09</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>2011-06</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>计算机科学与技术</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I11" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L11" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" s="7" t="str"/>
+      <x:c r="N11" s="6" t="str"/>
+      <x:c r="O11" s="6" t="str">
+        <x:v>本人明确2011 received B.E.。</x:v>
+      </x:c>
+      <x:c r="P11" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q11" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R11" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S11" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>2011-09</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>2017-12</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>计算机系统结构</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I12" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L12" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M12" s="7" t="str"/>
+      <x:c r="N12" s="6" t="str"/>
+      <x:c r="O12" s="6" t="str">
+        <x:v>本人明确2017 received Ph.D.；学习结束月不作授位月。</x:v>
+      </x:c>
+      <x:c r="P12" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q12" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R12" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S12" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str"/>
+      <x:c r="D13" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>2018-01</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>2021-03</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str"/>
+      <x:c r="H13" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I13" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L13" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="7" t="str"/>
+      <x:c r="N13" s="6" t="str"/>
+      <x:c r="O13" s="6" t="str"/>
+      <x:c r="P13" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q13" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R13" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S13" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>academic_visit</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str"/>
+      <x:c r="D14" s="6" t="str">
+        <x:v>伊利诺伊大学厄巴纳-香槟分校</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>2018-03</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>2018-06</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str"/>
+      <x:c r="H14" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I14" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K14" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L14" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="7" t="str"/>
+      <x:c r="N14" s="6" t="str"/>
+      <x:c r="O14" s="6" t="str"/>
+      <x:c r="P14" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q14" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R14" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S14" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>visiting_student</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str"/>
+      <x:c r="D15" s="6" t="str">
+        <x:v>弗吉尼亚联邦大学</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>2015-10</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>2016-04</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str"/>
+      <x:c r="H15" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I15" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K15" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L15" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="7" t="str"/>
+      <x:c r="N15" s="6" t="str"/>
+      <x:c r="O15" s="6" t="str"/>
+      <x:c r="P15" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q15" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R15" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S15" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>副研究员/副教授</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>华中科技大学计算机科学与技术学院</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str"/>
+      <x:c r="F16" s="6" t="str"/>
+      <x:c r="G16" s="6" t="str"/>
+      <x:c r="H16" s="6" t="str"/>
+      <x:c r="I16" s="6" t="str"/>
+      <x:c r="J16" s="6" t="str"/>
+      <x:c r="K16" s="6" t="str"/>
+      <x:c r="L16" s="6" t="str"/>
+      <x:c r="M16" s="7" t="str"/>
+      <x:c r="N16" s="6" t="str"/>
+      <x:c r="O16" s="6" t="str">
+        <x:v>同页头部Associate researcher、个人简介associate professor，原样冲突不自行选定。</x:v>
+      </x:c>
+      <x:c r="P16" s="6" t="str"/>
+      <x:c r="Q16" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="R16" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S16" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>College of Post and Telecommunication of WIT</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>2004-09</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>2008-06</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>计算机科学与技术（软件）</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I17" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K17" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L17" s="6" t="str"/>
+      <x:c r="M17" s="7" t="str"/>
+      <x:c r="N17" s="6" t="str"/>
+      <x:c r="O17" s="6" t="str">
+        <x:v>本人原文院校名保留，不能将独立学院等同武汉工程大学本部，历史法人/985属性待核。</x:v>
+      </x:c>
+      <x:c r="P17" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q17" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="R17" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S17" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>武汉工程大学</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="str">
+        <x:v>2008-09</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>2012-06</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
+        <x:v>模式识别与智能系统</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I18" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K18" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L18" s="6" t="str"/>
+      <x:c r="M18" s="7" t="str"/>
+      <x:c r="N18" s="6" t="str"/>
+      <x:c r="O18" s="6" t="str">
+        <x:v>仅学位学习标签；同段称three-year而区间近4年，保留原日期不修猜。</x:v>
+      </x:c>
+      <x:c r="P18" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q18" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="R18" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S18" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="str">
+        <x:v>2013-09</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str">
+        <x:v>2017-09</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="str">
+        <x:v>计算机系统结构</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I19" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J19" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K19" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L19" s="6" t="str"/>
+      <x:c r="M19" s="7" t="str"/>
+      <x:c r="N19" s="6" t="str"/>
+      <x:c r="O19" s="6" t="str">
+        <x:v>本人studied for doctorate并列学位标签，未独立明确获授。</x:v>
+      </x:c>
+      <x:c r="P19" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q19" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="R19" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S19" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="64" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str"/>
+      <x:c r="D20" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+      <x:c r="E20" s="6" t="str">
+        <x:v>2018-04</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str">
+        <x:v>2021-11</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="str">
+        <x:v>软件工程</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I20" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J20" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K20" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L20" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M20" s="7" t="str"/>
+      <x:c r="N20" s="6" t="str"/>
+      <x:c r="O20" s="6" t="str"/>
+      <x:c r="P20" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q20" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="R20" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S20" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="64" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>副研究员</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="str">
+        <x:v>华中科技大学计算机科学与技术学院</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="str">
+        <x:v>2021-12</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str"/>
+      <x:c r="G21" s="6" t="str"/>
+      <x:c r="H21" s="6" t="str"/>
+      <x:c r="I21" s="6" t="str"/>
+      <x:c r="J21" s="6" t="str"/>
+      <x:c r="K21" s="6" t="str"/>
+      <x:c r="L21" s="6" t="str"/>
+      <x:c r="M21" s="7" t="str"/>
+      <x:c r="N21" s="6" t="str"/>
+      <x:c r="O21" s="6" t="str">
+        <x:v>本人职业网页自述，校方名录对应身份；非人事在岗核验。</x:v>
+      </x:c>
+      <x:c r="P21" s="6" t="str"/>
+      <x:c r="Q21" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="R21" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="S21" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c02d32d15d4473"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76ad395cc9dd4e52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -882,8 +1720,203 @@
         <x:v>所属学校</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="64" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>Changsheng Xie</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>博士导师</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>本人明确博士指导教授，现职未知。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str"/>
+      <x:c r="H2" s="6" t="str"/>
+      <x:c r="I2" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str"/>
+      <x:c r="K2" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L2" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="64" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>Fei Wu</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>博士导师</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>本人明确博士指导教授，现职未知。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str"/>
+      <x:c r="H3" s="6" t="str"/>
+      <x:c r="I3" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str"/>
+      <x:c r="K3" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L3" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="64" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Yanduo Zhang</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>硕士导师</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>本人逐阶段明确Supervised by，现职未独立核。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str"/>
+      <x:c r="H4" s="6" t="str"/>
+      <x:c r="I4" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str"/>
+      <x:c r="K4" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>Ke Zhou</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>博士导师</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>本人逐阶段明确Supervised by，现职未独立核。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str"/>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L5" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>Fuhao Zou</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>博士导师</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>本人逐阶段明确Supervised by，现职未独立核。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str"/>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str"/>
+      <x:c r="K6" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L6" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>Ke Zhou</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>博士后合作导师（非学位授位导师）</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>本人逐阶段明确Supervised by，现职未独立核。 姓名按已直读英文原文，不猜中文对应。</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str"/>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str"/>
+      <x:c r="K7" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L7" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cf69bb8582f410f"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -979,10 +2012,118 @@
         <x:v>华中科技大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" ht="64" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>Reliable-Aware Clustering with Self-Ensemble Learning for Domain Adaptive Person Re-Identification</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str"/>
+      <x:c r="E3" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>期刊论文；journal_article</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="I3" s="6" t="str">
+        <x:v>仅官方精选书目已核，未逐篇核实出版社落地页或全文。；official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>官网精选列表，1527–1535；未逐篇出版者核。</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L3" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="64" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Remap-SSD: Safely and Efficiently Exploiting SSD Address Remapping to Eliminate Duplicate Writes</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str"/>
+      <x:c r="E4" s="6" t="str">
+        <x:v>https://www.usenix.org/conference/fast21/presentation/zhou</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>会议论文；conference_paper</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>https://www.usenix.org/conference/fast21/presentation/zhou</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="I4" s="6" t="str">
+        <x:v>出版社文章元数据已核，不表示全文已读。；article_metadata_verified</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>出版者直接列You Zhou和HUST，187–202。</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>FAVOR: Efficient Filter-Agnostic Vector ANNS Based on Selectivity-Aware Exclusion Distances</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str"/>
+      <x:c r="E5" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>期刊论文；journal_article</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="I5" s="6" t="str">
+        <x:v>仅本人职业网站所列书目，未核出版社落地页或全文。；self_authored_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>本人书目列4(3):183:1–183:25；未逐篇出版者核，不公开论文全文。</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="L5" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70ce6790389b4934"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4a256d9c5446e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1094,16 +2235,16 @@
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>张猛</x:v>
+        <x:v>陈加忠</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>institution-classification-3</x:v>
+        <x:v>chenjiazhong-source-1</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
-        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+        <x:v>https://cs.hust.edu.cn/szdw/jsml/ayjslb.htm</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+        <x:v>官方名录内容已读，仅保存本批选中观察。；official_roster_read</x:v>
       </x:c>
       <x:c r="E5" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
@@ -1112,13 +2253,312 @@
         <x:v>hust</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>chenjiazhong-source-2</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>https://faculty.hust.edu.cn/chenjiazhong/zh_CN/index.htm</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>目标读取超时，未取得该页正文。；timeout_not_read</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>chenjiazhong-source-3</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1565/1186.htm</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>官方公开正文已读，仅覆盖已审字段。；official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E7" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>zhouyou-source-1</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>https://cs.hust.edu.cn/szdw/jsml/ayjslb.htm</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>官方名录内容已读，仅保存本批选中观察。；official_roster_read</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>zhouyou-source-2</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>https://faculty.hust.edu.cn/zhouyou12/zh_CN/index.htm</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>目标读取超时，未取得该页正文。；timeout_not_read</x:v>
+      </x:c>
+      <x:c r="E9" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>zhouyou-source-3</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>https://en-cs.hust.edu.cn/info/1638/1547.htm</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>官方公开正文已读，仅覆盖已审字段。；official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E10" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>zhouyou-source-4</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>https://www.usenix.org/conference/fast21/presentation/zhou</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>出版社元数据已读，不表示全文已读。；publisher_metadata_read</x:v>
+      </x:c>
+      <x:c r="E11" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>liuyu-source-1</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>https://cs.hust.edu.cn/szdw/jsml/ayjslb.htm</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>官方名录内容已读，仅保存本批选中观察。；official_roster_read</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>liuyu-source-2</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>https://faculty.hust.edu.cn/liuyu123/zh_CN/index.htm</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>目标读取超时，未取得该页正文。；timeout_not_read</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>liuyu-source-3</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>https://lightyear416.github.io/liuyu/</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>本人公开职业网站自述，非学校门户正文或人事核验。；self_authored_professional_profile_read</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>张猛</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>institution-classification-3</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>陈加忠</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>institution-classification-3</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E16" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>周游</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>institution-classification-4</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>华中科技大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>刘渝</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>institution-classification-3</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>hust</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
         <x:v>华中科技大学</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87fccc4206da4478"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11a215626364aac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>